<commit_message>
Agrega 9 registros MET recuperados por el filtro corregido para revision
Border Fragment, Figure (315691-315696), Feathered Crown (315703), Feathered Ornament (316914) y Serpent ornament (316938) fueron excluidos por el filtro v1 por coincidencias por subcadena y penalizaciones de clasificacion mixta. Se agregan al workbook MET con corpus_final=revisar y metadatos del inventario; quedan en met_pendientes_revision_v2.csv (9) y en la galeria outputs/review/met_pendientes_revision_v2_galeria.html. El consolidado no cambia hasta la decision curatorial.
</commit_message>
<xml_diff>
--- a/data/metadata/met_revision_manual_v2.xlsx
+++ b/data/metadata/met_revision_manual_v2.xlsx
@@ -11,7 +11,7 @@
     <sheet name="listas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'revision_met_v2'!$A$1:$Z$212</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'revision_met_v2'!$A$1:$Z$221</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z212"/>
+  <dimension ref="A1:Z221"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19917,13 +19917,1017 @@
         </is>
       </c>
     </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>315691</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>recuperado_por_filtro_corregido</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Excluido por el filtro v1 (excluido_no_textil); el filtro corregido del 2026-10-05 lo clasifica como aceptado_textil (puntaje 11). Pendiente de revision visual.</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr"/>
+      <c r="H213" t="inlineStr"/>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>Border Fragment, Figure</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Fragmento textil</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>Nasca</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>2nd century BCE</t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="N213" t="inlineStr">
+        <is>
+          <t>borde_textil</t>
+        </is>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>borde_o_fragmento_lineal</t>
+        </is>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>Camelid hair</t>
+        </is>
+      </c>
+      <c r="Q213" t="inlineStr"/>
+      <c r="R213" t="inlineStr"/>
+      <c r="S213" t="inlineStr">
+        <is>
+          <t>pendiente_revision</t>
+        </is>
+      </c>
+      <c r="T213" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="U213" t="inlineStr">
+        <is>
+          <t>clasificación contiene evidencia textil: ['textiles'] | material contiene fibras o soporte textil: ['camelid'] | título contiene términos débiles asociados a fragmentos o paneles: ['fragment', 'border'] | evidencia cultural/geográfica andina: ['peru', 'nasca'] | clasificación mixta textil/no textil, sin penalización: ['sculpture'] | título con término no textil, sin penalización por evidencia textil: ['figure']</t>
+        </is>
+      </c>
+      <c r="V213" t="inlineStr">
+        <is>
+          <t>https://www.metmuseum.org/art/collection/search/315691</t>
+        </is>
+      </c>
+      <c r="W213" t="inlineStr">
+        <is>
+          <t>https://images.metmuseum.org/CRDImages/ao/original/DP18465.jpg</t>
+        </is>
+      </c>
+      <c r="X213" t="inlineStr"/>
+      <c r="Y213" t="inlineStr">
+        <is>
+          <t>Dominio público / Open Access según metadata de The Met</t>
+        </is>
+      </c>
+      <c r="Z213" t="inlineStr">
+        <is>
+          <t>recuperado_filtro_corregido</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>315692</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>recuperado_por_filtro_corregido</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Excluido por el filtro v1 (excluido_no_textil); el filtro corregido del 2026-10-05 lo clasifica como aceptado_textil (puntaje 11). Pendiente de revision visual.</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr"/>
+      <c r="H214" t="inlineStr"/>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Border Fragment, Figure</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>Fragmento textil</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>Nasca</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>2nd century BCE</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="N214" t="inlineStr">
+        <is>
+          <t>borde_textil</t>
+        </is>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>borde_o_fragmento_lineal</t>
+        </is>
+      </c>
+      <c r="P214" t="inlineStr">
+        <is>
+          <t>Camelid hair</t>
+        </is>
+      </c>
+      <c r="Q214" t="inlineStr"/>
+      <c r="R214" t="inlineStr"/>
+      <c r="S214" t="inlineStr">
+        <is>
+          <t>pendiente_revision</t>
+        </is>
+      </c>
+      <c r="T214" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="U214" t="inlineStr">
+        <is>
+          <t>clasificación contiene evidencia textil: ['textiles'] | material contiene fibras o soporte textil: ['camelid'] | título contiene términos débiles asociados a fragmentos o paneles: ['fragment', 'border'] | evidencia cultural/geográfica andina: ['peru', 'nasca'] | clasificación mixta textil/no textil, sin penalización: ['sculpture'] | título con término no textil, sin penalización por evidencia textil: ['figure']</t>
+        </is>
+      </c>
+      <c r="V214" t="inlineStr">
+        <is>
+          <t>https://www.metmuseum.org/art/collection/search/315692</t>
+        </is>
+      </c>
+      <c r="W214" t="inlineStr">
+        <is>
+          <t>https://images.metmuseum.org/CRDImages/ao/original/DP18467.jpg</t>
+        </is>
+      </c>
+      <c r="X214" t="inlineStr"/>
+      <c r="Y214" t="inlineStr">
+        <is>
+          <t>Dominio público / Open Access según metadata de The Met</t>
+        </is>
+      </c>
+      <c r="Z214" t="inlineStr">
+        <is>
+          <t>recuperado_filtro_corregido</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>315693</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>recuperado_por_filtro_corregido</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Excluido por el filtro v1 (excluido_no_textil); el filtro corregido del 2026-10-05 lo clasifica como aceptado_textil (puntaje 11). Pendiente de revision visual.</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr"/>
+      <c r="H215" t="inlineStr"/>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Border Fragment, Figure</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Fragmento textil</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>Nasca</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>2nd century BCE</t>
+        </is>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>borde_textil</t>
+        </is>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>borde_o_fragmento_lineal</t>
+        </is>
+      </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t>Camelid hair</t>
+        </is>
+      </c>
+      <c r="Q215" t="inlineStr"/>
+      <c r="R215" t="inlineStr"/>
+      <c r="S215" t="inlineStr">
+        <is>
+          <t>pendiente_revision</t>
+        </is>
+      </c>
+      <c r="T215" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="U215" t="inlineStr">
+        <is>
+          <t>clasificación contiene evidencia textil: ['textiles'] | material contiene fibras o soporte textil: ['camelid'] | título contiene términos débiles asociados a fragmentos o paneles: ['fragment', 'border'] | evidencia cultural/geográfica andina: ['peru', 'nasca'] | clasificación mixta textil/no textil, sin penalización: ['sculpture'] | título con término no textil, sin penalización por evidencia textil: ['figure']</t>
+        </is>
+      </c>
+      <c r="V215" t="inlineStr">
+        <is>
+          <t>https://www.metmuseum.org/art/collection/search/315693</t>
+        </is>
+      </c>
+      <c r="W215" t="inlineStr">
+        <is>
+          <t>https://images.metmuseum.org/CRDImages/ao/original/DP18470.jpg</t>
+        </is>
+      </c>
+      <c r="X215" t="inlineStr"/>
+      <c r="Y215" t="inlineStr">
+        <is>
+          <t>Dominio público / Open Access según metadata de The Met</t>
+        </is>
+      </c>
+      <c r="Z215" t="inlineStr">
+        <is>
+          <t>recuperado_filtro_corregido</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>315694</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>recuperado_por_filtro_corregido</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Excluido por el filtro v1 (excluido_no_textil); el filtro corregido del 2026-10-05 lo clasifica como aceptado_textil (puntaje 11). Pendiente de revision visual.</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr"/>
+      <c r="H216" t="inlineStr"/>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Border Fragment, Figure</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>Fragmento textil</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>Nasca</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>2nd century BCE</t>
+        </is>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="N216" t="inlineStr">
+        <is>
+          <t>borde_textil</t>
+        </is>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>borde_o_fragmento_lineal</t>
+        </is>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>Camelid hair</t>
+        </is>
+      </c>
+      <c r="Q216" t="inlineStr"/>
+      <c r="R216" t="inlineStr"/>
+      <c r="S216" t="inlineStr">
+        <is>
+          <t>pendiente_revision</t>
+        </is>
+      </c>
+      <c r="T216" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="U216" t="inlineStr">
+        <is>
+          <t>clasificación contiene evidencia textil: ['textiles'] | material contiene fibras o soporte textil: ['camelid'] | título contiene términos débiles asociados a fragmentos o paneles: ['fragment', 'border'] | evidencia cultural/geográfica andina: ['peru', 'nasca'] | clasificación mixta textil/no textil, sin penalización: ['sculpture'] | título con término no textil, sin penalización por evidencia textil: ['figure']</t>
+        </is>
+      </c>
+      <c r="V216" t="inlineStr">
+        <is>
+          <t>https://www.metmuseum.org/art/collection/search/315694</t>
+        </is>
+      </c>
+      <c r="W216" t="inlineStr">
+        <is>
+          <t>https://images.metmuseum.org/CRDImages/ao/original/DP18471.jpg</t>
+        </is>
+      </c>
+      <c r="X216" t="inlineStr"/>
+      <c r="Y216" t="inlineStr">
+        <is>
+          <t>Dominio público / Open Access según metadata de The Met</t>
+        </is>
+      </c>
+      <c r="Z216" t="inlineStr">
+        <is>
+          <t>recuperado_filtro_corregido</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>315695</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>recuperado_por_filtro_corregido</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Excluido por el filtro v1 (excluido_no_textil); el filtro corregido del 2026-10-05 lo clasifica como aceptado_textil (puntaje 11). Pendiente de revision visual.</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr"/>
+      <c r="H217" t="inlineStr"/>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Border Fragment, Figure</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Fragmento textil</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>Nasca</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>2nd century BCE</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="N217" t="inlineStr">
+        <is>
+          <t>borde_textil</t>
+        </is>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>borde_o_fragmento_lineal</t>
+        </is>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>Camelid hair</t>
+        </is>
+      </c>
+      <c r="Q217" t="inlineStr"/>
+      <c r="R217" t="inlineStr"/>
+      <c r="S217" t="inlineStr">
+        <is>
+          <t>pendiente_revision</t>
+        </is>
+      </c>
+      <c r="T217" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="U217" t="inlineStr">
+        <is>
+          <t>clasificación contiene evidencia textil: ['textiles'] | material contiene fibras o soporte textil: ['camelid'] | título contiene términos débiles asociados a fragmentos o paneles: ['fragment', 'border'] | evidencia cultural/geográfica andina: ['peru', 'nasca'] | clasificación mixta textil/no textil, sin penalización: ['sculpture'] | título con término no textil, sin penalización por evidencia textil: ['figure']</t>
+        </is>
+      </c>
+      <c r="V217" t="inlineStr">
+        <is>
+          <t>https://www.metmuseum.org/art/collection/search/315695</t>
+        </is>
+      </c>
+      <c r="W217" t="inlineStr">
+        <is>
+          <t>https://images.metmuseum.org/CRDImages/ao/original/DP18473.jpg</t>
+        </is>
+      </c>
+      <c r="X217" t="inlineStr"/>
+      <c r="Y217" t="inlineStr">
+        <is>
+          <t>Dominio público / Open Access según metadata de The Met</t>
+        </is>
+      </c>
+      <c r="Z217" t="inlineStr">
+        <is>
+          <t>recuperado_filtro_corregido</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>315696</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>recuperado_por_filtro_corregido</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Excluido por el filtro v1 (excluido_no_textil); el filtro corregido del 2026-10-05 lo clasifica como aceptado_textil (puntaje 11). Pendiente de revision visual.</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr"/>
+      <c r="H218" t="inlineStr"/>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Border Fragment, Figure</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>Fragmento textil</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>Nasca</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>2nd century BCE</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>borde_textil</t>
+        </is>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>borde_o_fragmento_lineal</t>
+        </is>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>Camelid hair</t>
+        </is>
+      </c>
+      <c r="Q218" t="inlineStr"/>
+      <c r="R218" t="inlineStr"/>
+      <c r="S218" t="inlineStr">
+        <is>
+          <t>pendiente_revision</t>
+        </is>
+      </c>
+      <c r="T218" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="U218" t="inlineStr">
+        <is>
+          <t>clasificación contiene evidencia textil: ['textiles'] | material contiene fibras o soporte textil: ['camelid'] | título contiene términos débiles asociados a fragmentos o paneles: ['fragment', 'border'] | evidencia cultural/geográfica andina: ['peru', 'nasca'] | clasificación mixta textil/no textil, sin penalización: ['sculpture'] | título con término no textil, sin penalización por evidencia textil: ['figure']</t>
+        </is>
+      </c>
+      <c r="V218" t="inlineStr">
+        <is>
+          <t>https://www.metmuseum.org/art/collection/search/315696</t>
+        </is>
+      </c>
+      <c r="W218" t="inlineStr">
+        <is>
+          <t>https://images.metmuseum.org/CRDImages/ao/original/DP18475.jpg</t>
+        </is>
+      </c>
+      <c r="X218" t="inlineStr"/>
+      <c r="Y218" t="inlineStr">
+        <is>
+          <t>Dominio público / Open Access según metadata de The Met</t>
+        </is>
+      </c>
+      <c r="Z218" t="inlineStr">
+        <is>
+          <t>recuperado_filtro_corregido</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>315703</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>recuperado_por_filtro_corregido</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Excluido por el filtro v1 (excluido_no_textil); el filtro corregido del 2026-10-05 lo clasifica como revision_manual (puntaje 5). Pendiente de revision visual.</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr"/>
+      <c r="H219" t="inlineStr"/>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Feathered Crown</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr"/>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>Chimú</t>
+        </is>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>1200 – 1400 CE</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="N219" t="inlineStr">
+        <is>
+          <t>tipo_no_determinado</t>
+        </is>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>revision_morfologica</t>
+        </is>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>Feathers (Paradise Tanager, Macaw), cotton, skin, cane, copper</t>
+        </is>
+      </c>
+      <c r="Q219" t="inlineStr"/>
+      <c r="R219" t="inlineStr"/>
+      <c r="S219" t="inlineStr">
+        <is>
+          <t>pendiente_revision</t>
+        </is>
+      </c>
+      <c r="T219" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="U219" t="inlineStr">
+        <is>
+          <t>material contiene fibras o soporte textil: ['cotton'] | evidencia cultural/geográfica andina: ['peru', 'chimú', 'chimu'] | material mixto con fibras textiles, sin penalización: ['copper']</t>
+        </is>
+      </c>
+      <c r="V219" t="inlineStr">
+        <is>
+          <t>https://www.metmuseum.org/art/collection/search/315703</t>
+        </is>
+      </c>
+      <c r="W219" t="inlineStr">
+        <is>
+          <t>https://images.metmuseum.org/CRDImages/ao/original/DP230213.jpg</t>
+        </is>
+      </c>
+      <c r="X219" t="inlineStr"/>
+      <c r="Y219" t="inlineStr">
+        <is>
+          <t>Dominio público / Open Access según metadata de The Met</t>
+        </is>
+      </c>
+      <c r="Z219" t="inlineStr">
+        <is>
+          <t>recuperado_filtro_corregido</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>316914</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>recuperado_por_filtro_corregido</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Excluido por el filtro v1 (excluido_no_textil); el filtro corregido del 2026-10-05 lo clasifica como aceptado_textil (puntaje 10). Pendiente de revision visual.</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr"/>
+      <c r="H220" t="inlineStr"/>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Feathered Ornament</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>Objeto textil</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>Peruvian</t>
+        </is>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>14th–early 16th century</t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>objeto_textil</t>
+        </is>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>superficie_amplia</t>
+        </is>
+      </c>
+      <c r="P220" t="inlineStr">
+        <is>
+          <t>Cotton, feathers</t>
+        </is>
+      </c>
+      <c r="Q220" t="inlineStr"/>
+      <c r="R220" t="inlineStr"/>
+      <c r="S220" t="inlineStr">
+        <is>
+          <t>pendiente_revision</t>
+        </is>
+      </c>
+      <c r="T220" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="U220" t="inlineStr">
+        <is>
+          <t>clasificación contiene evidencia textil: ['textiles'] | material contiene fibras o soporte textil: ['cotton'] | evidencia cultural/geográfica andina: ['peru', 'peruvian'] | título con término no textil, sin penalización por evidencia textil: ['ornament']</t>
+        </is>
+      </c>
+      <c r="V220" t="inlineStr">
+        <is>
+          <t>https://www.metmuseum.org/art/collection/search/316914</t>
+        </is>
+      </c>
+      <c r="W220" t="inlineStr">
+        <is>
+          <t>https://images.metmuseum.org/CRDImages/ao/original/DP101345b.jpg</t>
+        </is>
+      </c>
+      <c r="X220" t="inlineStr"/>
+      <c r="Y220" t="inlineStr">
+        <is>
+          <t>Dominio público / Open Access según metadata de The Met</t>
+        </is>
+      </c>
+      <c r="Z220" t="inlineStr">
+        <is>
+          <t>recuperado_filtro_corregido</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>316938</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>recuperado_por_filtro_corregido</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Excluido por el filtro v1 (excluido_no_textil); el filtro corregido del 2026-10-05 lo clasifica como aceptado_textil (puntaje 10). Pendiente de revision visual.</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr"/>
+      <c r="H221" t="inlineStr"/>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>Serpent ornament</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>Objeto textil</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>Inca (?)</t>
+        </is>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>1450–1532 CE</t>
+        </is>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="N221" t="inlineStr">
+        <is>
+          <t>objeto_textil</t>
+        </is>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>revision_morfologica</t>
+        </is>
+      </c>
+      <c r="P221" t="inlineStr">
+        <is>
+          <t>Cotton, camelid hair</t>
+        </is>
+      </c>
+      <c r="Q221" t="inlineStr"/>
+      <c r="R221" t="inlineStr"/>
+      <c r="S221" t="inlineStr">
+        <is>
+          <t>pendiente_revision</t>
+        </is>
+      </c>
+      <c r="T221" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="U221" t="inlineStr">
+        <is>
+          <t>clasificación contiene evidencia textil: ['textiles'] | material contiene fibras o soporte textil: ['cotton', 'camelid'] | evidencia cultural/geográfica andina: ['peru', 'inca'] | título con término no textil, sin penalización por evidencia textil: ['ornament']</t>
+        </is>
+      </c>
+      <c r="V221" t="inlineStr">
+        <is>
+          <t>https://www.metmuseum.org/art/collection/search/316938</t>
+        </is>
+      </c>
+      <c r="W221" t="inlineStr">
+        <is>
+          <t>https://images.metmuseum.org/CRDImages/ao/original/1994.35.113_d.JPG</t>
+        </is>
+      </c>
+      <c r="X221" t="inlineStr"/>
+      <c r="Y221" t="inlineStr">
+        <is>
+          <t>Dominio público / Open Access según metadata de The Met</t>
+        </is>
+      </c>
+      <c r="Z221" t="inlineStr">
+        <is>
+          <t>recuperado_filtro_corregido</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z212"/>
+  <autoFilter ref="A1:Z221"/>
   <dataValidations count="2">
-    <dataValidation sqref="C2:C212" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C2:C221" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"principal,secundario,descartados,revisar"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D212" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D2:D221" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"mantener,mover,descartar,recuperar,revisar"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Registra MET:307683 en principal y retira Excel prescindibles
- MET:307683: el revisor lo resuelve a principal porque sus colores y figuras se
  identifican (criterio v2); la validacion ciega lo habia dejado en revisar.
- Se retira el workbook de la curacion CMA v1 con sus dos scripts: sus
  decisiones estan completas en cma_corpus_*.csv, que sembraron el workbook v2.
- Se retira el xlsx de la auditoria MET v1, que duplicaba celda por celda su csv.
Ambos siguen en la etiqueta corpus-met-cma-v1.2 (docs/historico.md).
</commit_message>
<xml_diff>
--- a/data/metadata/met_revision_manual_v2.xlsx
+++ b/data/metadata/met_revision_manual_v2.xlsx
@@ -9804,12 +9804,12 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>revisar</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>revisar</t>
+          <t>mantener</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
@@ -9819,7 +9819,7 @@
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Anotación de la validación ciega del 2026-10-19 (data/metadata/validacion_met_cma_v2.xlsx, orden 4): descartados. Decisión anterior: principal (corpus_principal; superficie_textil_util). Queda en revisar: la anotación contradice su propio motivo según el criterio del 2026-10-19.</t>
+          <t>Anotación de la validación ciega del 2026-10-19 (data/metadata/validacion_met_cma_v2.xlsx, orden 4): descartados. Decisión anterior: principal (corpus_principal; superficie_textil_util). Queda en revisar: la anotación contradice su propio motivo según el criterio del 2026-10-19. Resuelto por el revisor el 2026-10-19: principal, porque sus colores y figuras se identifican (criterio v2).</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">

</xml_diff>